<commit_message>
Se añaden varios filtros para discriminar datos especificos para analisis de la información de las sedes educativas
</commit_message>
<xml_diff>
--- a/Sedes_a_priorizar_Nasa_CxaCxa.xlsx
+++ b/Sedes_a_priorizar_Nasa_CxaCxa.xlsx
@@ -450,7 +450,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B2" t="n">
         <v>219517800017</v>
@@ -481,7 +481,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B3" t="n">
         <v>219517001670</v>
@@ -512,7 +512,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B4" t="n">
         <v>219517000452</v>
@@ -543,7 +543,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B5" t="n">
         <v>219517000169</v>
@@ -574,7 +574,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B6" t="n">
         <v>219517000428</v>

</xml_diff>